<commit_message>
feat(bug hunting): added some test cases which helped to identify breaking EPC bugs
</commit_message>
<xml_diff>
--- a/docs/Raport_z_testow_gr3_zesp1.xlsx
+++ b/docs/Raport_z_testow_gr3_zesp1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nokia-my.sharepoint.com/personal/pawel_nogiec_nokia_com/Documents/szkolenia/Politechnika/testowanie_oprogramowania/gotowe/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nszyszka/Documents/studia/semestr_6/testowanie_oprogramowania/EPC/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="17" documentId="13_ncr:1_{88E62DB8-3785-4A14-8D67-BADFED2BF74F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CE5FE943-815E-0B45-A359-100488E7C2BD}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69FCFAE6-B008-BB40-B54E-29534888F70B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-25380" yWindow="900" windowWidth="35000" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Raport z testów" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="80">
   <si>
     <t>L.p.</t>
   </si>
@@ -122,14 +122,164 @@
     <t>Produkt:</t>
   </si>
   <si>
-    <t>Aplikacja bankomatu</t>
+    <t>Attach UE successfully</t>
+  </si>
+  <si>
+    <t>Attach UE with out of range ID</t>
+  </si>
+  <si>
+    <t>Attach already attached UE</t>
+  </si>
+  <si>
+    <t>Verify default bearer after attach</t>
+  </si>
+  <si>
+    <t>Detach UE successfully</t>
+  </si>
+  <si>
+    <t>Detach not attached UE</t>
+  </si>
+  <si>
+    <t>Stop traffic on specific bearer</t>
+  </si>
+  <si>
+    <t>Stop all traffic for UE</t>
+  </si>
+  <si>
+    <t>Stop traffic on non-existent bearer</t>
+  </si>
+  <si>
+    <t>Add bearer successfully</t>
+  </si>
+  <si>
+    <t>Add bearer out of range</t>
+  </si>
+  <si>
+    <t>Add already existing bearer</t>
+  </si>
+  <si>
+    <t>Start traffic successfully</t>
+  </si>
+  <si>
+    <t>Start traffic with out of range speed</t>
+  </si>
+  <si>
+    <t>Start traffic on non-existent bearer</t>
+  </si>
+  <si>
+    <t>Get connected bearers successfully</t>
+  </si>
+  <si>
+    <t>Get connected bearers for non-existent UE</t>
+  </si>
+  <si>
+    <t>Get bearer transfer stats with no traffic</t>
+  </si>
+  <si>
+    <t>Get bearer transfer after starting traffic</t>
+  </si>
+  <si>
+    <t>Get aggregated transfer stats with no traffic</t>
+  </si>
+  <si>
+    <t>Get aggregated transfer with one active bearer</t>
+  </si>
+  <si>
+    <t>Get aggregated transfer with multiple bearers</t>
+  </si>
+  <si>
+    <t>Get aggregated transfer details per bearer</t>
+  </si>
+  <si>
+    <t>Get aggregated transfer for non-existent UE</t>
+  </si>
+  <si>
+    <t>Get global transfer stat</t>
+  </si>
+  <si>
+    <t>Delete dedicated bearer successfully</t>
+  </si>
+  <si>
+    <t>Delete bearer removes it from UE bearer list</t>
+  </si>
+  <si>
+    <t>Cannot delete default beare</t>
+  </si>
+  <si>
+    <t>Delete bearer out of range</t>
+  </si>
+  <si>
+    <t>Delete inactive bearer not on UE</t>
+  </si>
+  <si>
+    <t>Delete bearer twice fails</t>
+  </si>
+  <si>
+    <t>Delete bearer when UE not found</t>
+  </si>
+  <si>
+    <t>UE ID 0 should be valid per spec range 0-100</t>
+  </si>
+  <si>
+    <t>Start traffic with negative speed rejected</t>
+  </si>
+  <si>
+    <t>Start traffic with zero speed rejected</t>
+  </si>
+  <si>
+    <t>Get transfer stats for bearer not on UE returns error</t>
+  </si>
+  <si>
+    <t>Traffic stats unit parameter should affect returned values</t>
+  </si>
+  <si>
+    <t>Start traffic twice on same bearer fails</t>
+  </si>
+  <si>
+    <t>Stop traffic with no active transfer returns error</t>
+  </si>
+  <si>
+    <t>Traffic is downlink only</t>
+  </si>
+  <si>
+    <t>Delete bearer with active traffic rejected</t>
+  </si>
+  <si>
+    <t>Attach UE with string ID rejected</t>
+  </si>
+  <si>
+    <t>Add bearer with string ID rejected</t>
+  </si>
+  <si>
+    <t>Detach UE with active traffic rejected</t>
+  </si>
+  <si>
+    <t>Attach UE with boolean ID rejected</t>
+  </si>
+  <si>
+    <t>Add bearer with boolean ID rejected</t>
+  </si>
+  <si>
+    <t>Start traffic with string kbps rejected</t>
+  </si>
+  <si>
+    <t>Deleting bearer should stop its traffic stats from being available</t>
+  </si>
+  <si>
+    <t>Stop traffic twice should fail second time</t>
+  </si>
+  <si>
+    <t>Evolved Packet Core - EPC simulator</t>
+  </si>
+  <si>
+    <t>niepoprawne</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -154,13 +304,6 @@
       <family val="2"/>
     </font>
     <font>
-      <u/>
-      <sz val="10"/>
-      <color rgb="FF1155CC"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="10"/>
       <color rgb="FFFF0000"/>
       <name val="Arial"/>
@@ -182,8 +325,44 @@
       <charset val="238"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF1155CC"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -211,6 +390,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
   </fills>
@@ -351,49 +536,43 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="10" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="10" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -403,12 +582,1148 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Calculation" xfId="1" builtinId="22"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="5">
+  <dxfs count="160">
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color auto="1"/>
@@ -659,14 +1974,14 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
-  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:K53"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="9.453125" customWidth="1"/>
-    <col min="3" max="3" width="56.81640625" customWidth="1"/>
+    <col min="1" max="1" width="9.5" customWidth="1"/>
+    <col min="3" max="3" width="56.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="32.5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="33" x14ac:dyDescent="0.15">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="2" t="s">
@@ -679,13 +1994,13 @@
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
     </row>
-    <row r="2" spans="1:9" ht="14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" ht="14" x14ac:dyDescent="0.15">
       <c r="A2" s="1"/>
       <c r="B2" s="1" t="s">
         <v>28</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>29</v>
+        <v>78</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -694,7 +2009,7 @@
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
     </row>
-    <row r="3" spans="1:9" ht="14" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" ht="14" x14ac:dyDescent="0.15">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -705,7 +2020,7 @@
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
     </row>
-    <row r="4" spans="1:9" ht="28" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" ht="30" x14ac:dyDescent="0.15">
       <c r="A4" s="12" t="s">
         <v>0</v>
       </c>
@@ -734,97 +2049,1279 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="14" x14ac:dyDescent="0.3">
-      <c r="A5" s="13">
+    <row r="5" spans="1:11" ht="15" x14ac:dyDescent="0.2">
+      <c r="A5" s="23">
         <v>1</v>
       </c>
-      <c r="B5" s="14"/>
-      <c r="C5" s="15"/>
+      <c r="B5" s="24">
+        <v>1</v>
+      </c>
+      <c r="C5" s="20" t="s">
+        <v>29</v>
+      </c>
       <c r="D5" s="13"/>
-      <c r="E5" s="13" t="s">
+      <c r="E5" s="23" t="s">
+        <v>8</v>
+      </c>
+      <c r="F5" s="13"/>
+      <c r="G5" s="14"/>
+      <c r="H5" s="14"/>
+      <c r="I5" s="15"/>
+      <c r="K5" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="13"/>
-      <c r="G5" s="15"/>
-      <c r="H5" s="15"/>
-      <c r="I5" s="16"/>
-    </row>
-    <row r="6" spans="1:9" ht="14" x14ac:dyDescent="0.3">
-      <c r="A6" s="13">
+    </row>
+    <row r="6" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="A6" s="23">
         <v>2</v>
       </c>
-      <c r="B6" s="14"/>
-      <c r="C6" s="17"/>
+      <c r="B6" s="24">
+        <v>2</v>
+      </c>
+      <c r="C6" s="21" t="s">
+        <v>30</v>
+      </c>
       <c r="D6" s="13"/>
-      <c r="E6" s="13" t="s">
+      <c r="E6" s="23" t="s">
         <v>8</v>
       </c>
       <c r="F6" s="13"/>
-      <c r="G6" s="15"/>
-      <c r="H6" s="15"/>
-      <c r="I6" s="16"/>
-    </row>
-    <row r="7" spans="1:9" ht="14" x14ac:dyDescent="0.3">
-      <c r="A7" s="13">
+      <c r="G6" s="14"/>
+      <c r="H6" s="14"/>
+      <c r="I6" s="15"/>
+      <c r="K6" s="23" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="15" x14ac:dyDescent="0.2">
+      <c r="A7" s="23">
         <v>3</v>
       </c>
-      <c r="B7" s="14"/>
-      <c r="C7" s="17"/>
-      <c r="D7" s="16"/>
-      <c r="E7" s="13" t="s">
+      <c r="B7" s="24">
+        <v>3</v>
+      </c>
+      <c r="C7" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" s="15"/>
+      <c r="E7" s="23" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" s="13"/>
+      <c r="G7" s="14"/>
+      <c r="H7" s="14"/>
+      <c r="I7" s="15"/>
+      <c r="K7" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="F7" s="13"/>
-      <c r="G7" s="15"/>
-      <c r="H7" s="15"/>
-      <c r="I7" s="16"/>
-    </row>
-    <row r="8" spans="1:9" ht="14" x14ac:dyDescent="0.3">
-      <c r="A8" s="13">
+    </row>
+    <row r="8" spans="1:11" ht="15" x14ac:dyDescent="0.2">
+      <c r="A8" s="23">
         <v>4</v>
       </c>
-      <c r="B8" s="14"/>
-      <c r="C8" s="17"/>
+      <c r="B8" s="24">
+        <v>4</v>
+      </c>
+      <c r="C8" s="22" t="s">
+        <v>32</v>
+      </c>
       <c r="D8" s="13"/>
-      <c r="E8" s="13" t="s">
+      <c r="E8" s="23" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" s="13"/>
+      <c r="G8" s="14"/>
+      <c r="H8" s="14"/>
+      <c r="I8" s="15"/>
+      <c r="K8" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="F8" s="13"/>
-      <c r="G8" s="15"/>
-      <c r="H8" s="15"/>
-      <c r="I8" s="16"/>
-    </row>
-    <row r="9" spans="1:9" ht="14" x14ac:dyDescent="0.3">
-      <c r="A9" s="13">
+    </row>
+    <row r="9" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="A9" s="23">
         <v>5</v>
       </c>
-      <c r="B9" s="14"/>
-      <c r="C9" s="17"/>
-      <c r="D9" s="16"/>
-      <c r="E9" s="13" t="s">
+      <c r="B9" s="24">
+        <v>5</v>
+      </c>
+      <c r="C9" s="21" t="s">
+        <v>33</v>
+      </c>
+      <c r="D9" s="15"/>
+      <c r="E9" s="23" t="s">
+        <v>8</v>
+      </c>
+      <c r="F9" s="13"/>
+      <c r="G9" s="14"/>
+      <c r="H9" s="14"/>
+      <c r="I9" s="15"/>
+      <c r="K9" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="F9" s="13"/>
-      <c r="G9" s="15"/>
-      <c r="H9" s="15"/>
-      <c r="I9" s="16"/>
+    </row>
+    <row r="10" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="23">
+        <v>6</v>
+      </c>
+      <c r="B10" s="24">
+        <v>6</v>
+      </c>
+      <c r="C10" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="E10" s="23" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="23">
+        <v>7</v>
+      </c>
+      <c r="B11" s="24">
+        <v>7</v>
+      </c>
+      <c r="C11" s="22" t="s">
+        <v>35</v>
+      </c>
+      <c r="E11" s="23" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="23">
+        <v>8</v>
+      </c>
+      <c r="B12" s="24">
+        <v>8</v>
+      </c>
+      <c r="C12" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="E12" s="23" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="23">
+        <v>9</v>
+      </c>
+      <c r="B13" s="24">
+        <v>9</v>
+      </c>
+      <c r="C13" s="22" t="s">
+        <v>37</v>
+      </c>
+      <c r="E13" s="23" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="23">
+        <v>10</v>
+      </c>
+      <c r="B14" s="24">
+        <v>10</v>
+      </c>
+      <c r="C14" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="E14" s="23" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="23">
+        <v>11</v>
+      </c>
+      <c r="B15" s="24">
+        <v>11</v>
+      </c>
+      <c r="C15" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="E15" s="23" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="23">
+        <v>12</v>
+      </c>
+      <c r="B16" s="24">
+        <v>12</v>
+      </c>
+      <c r="C16" s="22" t="s">
+        <v>40</v>
+      </c>
+      <c r="E16" s="23" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="23">
+        <v>13</v>
+      </c>
+      <c r="B17" s="24">
+        <v>13</v>
+      </c>
+      <c r="C17" s="22" t="s">
+        <v>41</v>
+      </c>
+      <c r="E17" s="23" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="23">
+        <v>14</v>
+      </c>
+      <c r="B18" s="24">
+        <v>14</v>
+      </c>
+      <c r="C18" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="E18" s="23" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="23">
+        <v>15</v>
+      </c>
+      <c r="B19" s="24">
+        <v>15</v>
+      </c>
+      <c r="C19" s="22" t="s">
+        <v>43</v>
+      </c>
+      <c r="E19" s="25" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="23">
+        <v>16</v>
+      </c>
+      <c r="B20" s="24">
+        <v>16</v>
+      </c>
+      <c r="C20" s="22" t="s">
+        <v>44</v>
+      </c>
+      <c r="E20" s="25" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="23">
+        <v>17</v>
+      </c>
+      <c r="B21" s="24">
+        <v>17</v>
+      </c>
+      <c r="C21" s="22" t="s">
+        <v>45</v>
+      </c>
+      <c r="E21" s="25" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="23">
+        <v>18</v>
+      </c>
+      <c r="B22" s="24">
+        <v>18</v>
+      </c>
+      <c r="C22" s="22" t="s">
+        <v>46</v>
+      </c>
+      <c r="E22" s="25" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="23">
+        <v>19</v>
+      </c>
+      <c r="B23" s="24">
+        <v>19</v>
+      </c>
+      <c r="C23" s="22" t="s">
+        <v>47</v>
+      </c>
+      <c r="E23" s="25" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="23">
+        <v>20</v>
+      </c>
+      <c r="B24" s="24">
+        <v>20</v>
+      </c>
+      <c r="C24" s="22" t="s">
+        <v>48</v>
+      </c>
+      <c r="E24" s="25" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="23">
+        <v>21</v>
+      </c>
+      <c r="B25" s="24">
+        <v>21</v>
+      </c>
+      <c r="C25" s="22" t="s">
+        <v>49</v>
+      </c>
+      <c r="E25" s="25" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="23">
+        <v>22</v>
+      </c>
+      <c r="B26" s="24">
+        <v>22</v>
+      </c>
+      <c r="C26" s="22" t="s">
+        <v>50</v>
+      </c>
+      <c r="E26" s="25" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="23">
+        <v>23</v>
+      </c>
+      <c r="B27" s="24">
+        <v>23</v>
+      </c>
+      <c r="C27" s="22" t="s">
+        <v>51</v>
+      </c>
+      <c r="E27" s="25" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="23">
+        <v>24</v>
+      </c>
+      <c r="B28" s="24">
+        <v>24</v>
+      </c>
+      <c r="C28" s="22" t="s">
+        <v>52</v>
+      </c>
+      <c r="E28" s="25" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="23">
+        <v>25</v>
+      </c>
+      <c r="B29" s="24">
+        <v>25</v>
+      </c>
+      <c r="C29" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="E29" s="25" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="23">
+        <v>26</v>
+      </c>
+      <c r="B30" s="24">
+        <v>26</v>
+      </c>
+      <c r="C30" s="22" t="s">
+        <v>54</v>
+      </c>
+      <c r="E30" s="25" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="23">
+        <v>27</v>
+      </c>
+      <c r="B31" s="24">
+        <v>27</v>
+      </c>
+      <c r="C31" s="22" t="s">
+        <v>55</v>
+      </c>
+      <c r="E31" s="25" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="23">
+        <v>28</v>
+      </c>
+      <c r="B32" s="24">
+        <v>28</v>
+      </c>
+      <c r="C32" s="22" t="s">
+        <v>56</v>
+      </c>
+      <c r="E32" s="25" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="23">
+        <v>29</v>
+      </c>
+      <c r="B33" s="24">
+        <v>29</v>
+      </c>
+      <c r="C33" s="22" t="s">
+        <v>57</v>
+      </c>
+      <c r="E33" s="25" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="23">
+        <v>30</v>
+      </c>
+      <c r="B34" s="24">
+        <v>30</v>
+      </c>
+      <c r="C34" s="22" t="s">
+        <v>58</v>
+      </c>
+      <c r="E34" s="25" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="23">
+        <v>31</v>
+      </c>
+      <c r="B35" s="24">
+        <v>31</v>
+      </c>
+      <c r="C35" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="E35" s="25" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="23">
+        <v>32</v>
+      </c>
+      <c r="B36" s="24">
+        <v>32</v>
+      </c>
+      <c r="C36" s="22" t="s">
+        <v>60</v>
+      </c>
+      <c r="E36" s="25" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="23">
+        <v>33</v>
+      </c>
+      <c r="B37" s="24">
+        <v>33</v>
+      </c>
+      <c r="C37" s="22" t="s">
+        <v>61</v>
+      </c>
+      <c r="E37" s="23" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="23">
+        <v>34</v>
+      </c>
+      <c r="B38" s="24">
+        <v>34</v>
+      </c>
+      <c r="C38" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="E38" s="23" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="23">
+        <v>35</v>
+      </c>
+      <c r="B39" s="24">
+        <v>35</v>
+      </c>
+      <c r="C39" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="E39" s="23" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="23">
+        <v>36</v>
+      </c>
+      <c r="B40" s="24">
+        <v>36</v>
+      </c>
+      <c r="C40" s="22" t="s">
+        <v>64</v>
+      </c>
+      <c r="E40" s="23" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="23">
+        <v>37</v>
+      </c>
+      <c r="B41" s="24">
+        <v>37</v>
+      </c>
+      <c r="C41" s="22" t="s">
+        <v>65</v>
+      </c>
+      <c r="E41" s="23" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="23">
+        <v>38</v>
+      </c>
+      <c r="B42" s="24">
+        <v>38</v>
+      </c>
+      <c r="C42" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="E42" s="25" t="s">
+        <v>8</v>
+      </c>
+      <c r="I42" s="26" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="23">
+        <v>39</v>
+      </c>
+      <c r="B43" s="24">
+        <v>39</v>
+      </c>
+      <c r="C43" s="22" t="s">
+        <v>67</v>
+      </c>
+      <c r="E43" s="23" t="s">
+        <v>10</v>
+      </c>
+      <c r="I43" s="19"/>
+    </row>
+    <row r="44" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="23">
+        <v>40</v>
+      </c>
+      <c r="B44" s="24">
+        <v>40</v>
+      </c>
+      <c r="C44" s="22" t="s">
+        <v>68</v>
+      </c>
+      <c r="E44" s="23" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="23">
+        <v>41</v>
+      </c>
+      <c r="B45" s="24">
+        <v>41</v>
+      </c>
+      <c r="C45" s="22" t="s">
+        <v>69</v>
+      </c>
+      <c r="E45" s="23" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="23">
+        <v>42</v>
+      </c>
+      <c r="B46" s="24">
+        <v>42</v>
+      </c>
+      <c r="C46" s="22" t="s">
+        <v>70</v>
+      </c>
+      <c r="E46" s="23" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A47" s="23">
+        <v>43</v>
+      </c>
+      <c r="B47" s="24">
+        <v>43</v>
+      </c>
+      <c r="C47" s="22" t="s">
+        <v>71</v>
+      </c>
+      <c r="E47" s="23" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A48" s="23">
+        <v>44</v>
+      </c>
+      <c r="B48" s="24">
+        <v>44</v>
+      </c>
+      <c r="C48" s="22" t="s">
+        <v>72</v>
+      </c>
+      <c r="E48" s="23" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A49" s="23">
+        <v>45</v>
+      </c>
+      <c r="B49" s="24">
+        <v>45</v>
+      </c>
+      <c r="C49" s="22" t="s">
+        <v>73</v>
+      </c>
+      <c r="E49" s="23" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A50" s="23">
+        <v>46</v>
+      </c>
+      <c r="B50" s="24">
+        <v>46</v>
+      </c>
+      <c r="C50" s="22" t="s">
+        <v>74</v>
+      </c>
+      <c r="E50" s="23" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="23">
+        <v>47</v>
+      </c>
+      <c r="B51" s="24">
+        <v>47</v>
+      </c>
+      <c r="C51" s="22" t="s">
+        <v>75</v>
+      </c>
+      <c r="E51" s="23" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A52" s="23">
+        <v>48</v>
+      </c>
+      <c r="B52" s="24">
+        <v>48</v>
+      </c>
+      <c r="C52" s="22" t="s">
+        <v>76</v>
+      </c>
+      <c r="E52" s="23" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A53" s="23">
+        <v>49</v>
+      </c>
+      <c r="B53" s="24">
+        <v>49</v>
+      </c>
+      <c r="C53" s="22" t="s">
+        <v>77</v>
+      </c>
+      <c r="E53" s="23" t="s">
+        <v>10</v>
+      </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="E5:F9">
+  <conditionalFormatting sqref="F5:F9">
+    <cfRule type="containsText" dxfId="159" priority="156" operator="containsText" text="no run">
+      <formula>NOT(ISERROR(SEARCH("no run",F5)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="158" priority="157" operator="containsText" text="blocked">
+      <formula>NOT(ISERROR(SEARCH("blocked",F5)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="157" priority="158" operator="containsText" text="in progres">
+      <formula>NOT(ISERROR(SEARCH("in progres",F5)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="156" priority="159" operator="containsText" text="failed">
+      <formula>NOT(ISERROR(SEARCH("failed",F5)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="155" priority="160" operator="containsText" text="passed">
+      <formula>NOT(ISERROR(SEARCH("passed",F5)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K5:K9">
+    <cfRule type="containsText" dxfId="154" priority="151" operator="containsText" text="no run">
+      <formula>NOT(ISERROR(SEARCH("no run",K5)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="153" priority="152" operator="containsText" text="blocked">
+      <formula>NOT(ISERROR(SEARCH("blocked",K5)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="152" priority="153" operator="containsText" text="in progres">
+      <formula>NOT(ISERROR(SEARCH("in progres",K5)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="151" priority="154" operator="containsText" text="failed">
+      <formula>NOT(ISERROR(SEARCH("failed",K5)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="150" priority="155" operator="containsText" text="passed">
+      <formula>NOT(ISERROR(SEARCH("passed",K5)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E5">
+    <cfRule type="containsText" dxfId="149" priority="146" operator="containsText" text="no run">
+      <formula>NOT(ISERROR(SEARCH("no run",E5)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="148" priority="147" operator="containsText" text="blocked">
+      <formula>NOT(ISERROR(SEARCH("blocked",E5)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="147" priority="148" operator="containsText" text="in progres">
+      <formula>NOT(ISERROR(SEARCH("in progres",E5)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="146" priority="149" operator="containsText" text="failed">
+      <formula>NOT(ISERROR(SEARCH("failed",E5)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="145" priority="150" operator="containsText" text="passed">
+      <formula>NOT(ISERROR(SEARCH("passed",E5)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E6">
+    <cfRule type="containsText" dxfId="144" priority="141" operator="containsText" text="no run">
+      <formula>NOT(ISERROR(SEARCH("no run",E6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="143" priority="142" operator="containsText" text="blocked">
+      <formula>NOT(ISERROR(SEARCH("blocked",E6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="142" priority="143" operator="containsText" text="in progres">
+      <formula>NOT(ISERROR(SEARCH("in progres",E6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="141" priority="144" operator="containsText" text="failed">
+      <formula>NOT(ISERROR(SEARCH("failed",E6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="140" priority="145" operator="containsText" text="passed">
+      <formula>NOT(ISERROR(SEARCH("passed",E6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E7">
+    <cfRule type="containsText" dxfId="139" priority="136" operator="containsText" text="no run">
+      <formula>NOT(ISERROR(SEARCH("no run",E7)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="138" priority="137" operator="containsText" text="blocked">
+      <formula>NOT(ISERROR(SEARCH("blocked",E7)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="137" priority="138" operator="containsText" text="in progres">
+      <formula>NOT(ISERROR(SEARCH("in progres",E7)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="136" priority="139" operator="containsText" text="failed">
+      <formula>NOT(ISERROR(SEARCH("failed",E7)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="135" priority="140" operator="containsText" text="passed">
+      <formula>NOT(ISERROR(SEARCH("passed",E7)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E8">
+    <cfRule type="containsText" dxfId="134" priority="131" operator="containsText" text="no run">
+      <formula>NOT(ISERROR(SEARCH("no run",E8)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="133" priority="132" operator="containsText" text="blocked">
+      <formula>NOT(ISERROR(SEARCH("blocked",E8)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="132" priority="133" operator="containsText" text="in progres">
+      <formula>NOT(ISERROR(SEARCH("in progres",E8)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="131" priority="134" operator="containsText" text="failed">
+      <formula>NOT(ISERROR(SEARCH("failed",E8)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="130" priority="135" operator="containsText" text="passed">
+      <formula>NOT(ISERROR(SEARCH("passed",E8)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E9">
+    <cfRule type="containsText" dxfId="129" priority="126" operator="containsText" text="no run">
+      <formula>NOT(ISERROR(SEARCH("no run",E9)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="128" priority="127" operator="containsText" text="blocked">
+      <formula>NOT(ISERROR(SEARCH("blocked",E9)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="127" priority="128" operator="containsText" text="in progres">
+      <formula>NOT(ISERROR(SEARCH("in progres",E9)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="126" priority="129" operator="containsText" text="failed">
+      <formula>NOT(ISERROR(SEARCH("failed",E9)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="125" priority="130" operator="containsText" text="passed">
+      <formula>NOT(ISERROR(SEARCH("passed",E9)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E10">
+    <cfRule type="containsText" dxfId="124" priority="121" operator="containsText" text="no run">
+      <formula>NOT(ISERROR(SEARCH("no run",E10)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="123" priority="122" operator="containsText" text="blocked">
+      <formula>NOT(ISERROR(SEARCH("blocked",E10)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="122" priority="123" operator="containsText" text="in progres">
+      <formula>NOT(ISERROR(SEARCH("in progres",E10)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="121" priority="124" operator="containsText" text="failed">
+      <formula>NOT(ISERROR(SEARCH("failed",E10)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="120" priority="125" operator="containsText" text="passed">
+      <formula>NOT(ISERROR(SEARCH("passed",E10)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E11">
+    <cfRule type="containsText" dxfId="119" priority="116" operator="containsText" text="no run">
+      <formula>NOT(ISERROR(SEARCH("no run",E11)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="118" priority="117" operator="containsText" text="blocked">
+      <formula>NOT(ISERROR(SEARCH("blocked",E11)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="117" priority="118" operator="containsText" text="in progres">
+      <formula>NOT(ISERROR(SEARCH("in progres",E11)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="116" priority="119" operator="containsText" text="failed">
+      <formula>NOT(ISERROR(SEARCH("failed",E11)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="115" priority="120" operator="containsText" text="passed">
+      <formula>NOT(ISERROR(SEARCH("passed",E11)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E12">
+    <cfRule type="containsText" dxfId="114" priority="111" operator="containsText" text="no run">
+      <formula>NOT(ISERROR(SEARCH("no run",E12)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="113" priority="112" operator="containsText" text="blocked">
+      <formula>NOT(ISERROR(SEARCH("blocked",E12)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="112" priority="113" operator="containsText" text="in progres">
+      <formula>NOT(ISERROR(SEARCH("in progres",E12)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="111" priority="114" operator="containsText" text="failed">
+      <formula>NOT(ISERROR(SEARCH("failed",E12)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="110" priority="115" operator="containsText" text="passed">
+      <formula>NOT(ISERROR(SEARCH("passed",E12)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E13">
+    <cfRule type="containsText" dxfId="109" priority="106" operator="containsText" text="no run">
+      <formula>NOT(ISERROR(SEARCH("no run",E13)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="108" priority="107" operator="containsText" text="blocked">
+      <formula>NOT(ISERROR(SEARCH("blocked",E13)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="107" priority="108" operator="containsText" text="in progres">
+      <formula>NOT(ISERROR(SEARCH("in progres",E13)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="106" priority="109" operator="containsText" text="failed">
+      <formula>NOT(ISERROR(SEARCH("failed",E13)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="105" priority="110" operator="containsText" text="passed">
+      <formula>NOT(ISERROR(SEARCH("passed",E13)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E14">
+    <cfRule type="containsText" dxfId="104" priority="101" operator="containsText" text="no run">
+      <formula>NOT(ISERROR(SEARCH("no run",E14)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="103" priority="102" operator="containsText" text="blocked">
+      <formula>NOT(ISERROR(SEARCH("blocked",E14)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="102" priority="103" operator="containsText" text="in progres">
+      <formula>NOT(ISERROR(SEARCH("in progres",E14)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="101" priority="104" operator="containsText" text="failed">
+      <formula>NOT(ISERROR(SEARCH("failed",E14)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="100" priority="105" operator="containsText" text="passed">
+      <formula>NOT(ISERROR(SEARCH("passed",E14)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E15">
+    <cfRule type="containsText" dxfId="99" priority="96" operator="containsText" text="no run">
+      <formula>NOT(ISERROR(SEARCH("no run",E15)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="98" priority="97" operator="containsText" text="blocked">
+      <formula>NOT(ISERROR(SEARCH("blocked",E15)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="97" priority="98" operator="containsText" text="in progres">
+      <formula>NOT(ISERROR(SEARCH("in progres",E15)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="96" priority="99" operator="containsText" text="failed">
+      <formula>NOT(ISERROR(SEARCH("failed",E15)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="95" priority="100" operator="containsText" text="passed">
+      <formula>NOT(ISERROR(SEARCH("passed",E15)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E16">
+    <cfRule type="containsText" dxfId="94" priority="91" operator="containsText" text="no run">
+      <formula>NOT(ISERROR(SEARCH("no run",E16)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="93" priority="92" operator="containsText" text="blocked">
+      <formula>NOT(ISERROR(SEARCH("blocked",E16)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="92" priority="93" operator="containsText" text="in progres">
+      <formula>NOT(ISERROR(SEARCH("in progres",E16)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="91" priority="94" operator="containsText" text="failed">
+      <formula>NOT(ISERROR(SEARCH("failed",E16)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="90" priority="95" operator="containsText" text="passed">
+      <formula>NOT(ISERROR(SEARCH("passed",E16)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E17">
+    <cfRule type="containsText" dxfId="89" priority="86" operator="containsText" text="no run">
+      <formula>NOT(ISERROR(SEARCH("no run",E17)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="88" priority="87" operator="containsText" text="blocked">
+      <formula>NOT(ISERROR(SEARCH("blocked",E17)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="87" priority="88" operator="containsText" text="in progres">
+      <formula>NOT(ISERROR(SEARCH("in progres",E17)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="86" priority="89" operator="containsText" text="failed">
+      <formula>NOT(ISERROR(SEARCH("failed",E17)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="85" priority="90" operator="containsText" text="passed">
+      <formula>NOT(ISERROR(SEARCH("passed",E17)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E18">
+    <cfRule type="containsText" dxfId="84" priority="81" operator="containsText" text="no run">
+      <formula>NOT(ISERROR(SEARCH("no run",E18)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="83" priority="82" operator="containsText" text="blocked">
+      <formula>NOT(ISERROR(SEARCH("blocked",E18)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="82" priority="83" operator="containsText" text="in progres">
+      <formula>NOT(ISERROR(SEARCH("in progres",E18)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="81" priority="84" operator="containsText" text="failed">
+      <formula>NOT(ISERROR(SEARCH("failed",E18)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="80" priority="85" operator="containsText" text="passed">
+      <formula>NOT(ISERROR(SEARCH("passed",E18)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E37">
+    <cfRule type="containsText" dxfId="79" priority="76" operator="containsText" text="no run">
+      <formula>NOT(ISERROR(SEARCH("no run",E37)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="78" priority="77" operator="containsText" text="blocked">
+      <formula>NOT(ISERROR(SEARCH("blocked",E37)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="77" priority="78" operator="containsText" text="in progres">
+      <formula>NOT(ISERROR(SEARCH("in progres",E37)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="76" priority="79" operator="containsText" text="failed">
+      <formula>NOT(ISERROR(SEARCH("failed",E37)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="75" priority="80" operator="containsText" text="passed">
+      <formula>NOT(ISERROR(SEARCH("passed",E37)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E38">
+    <cfRule type="containsText" dxfId="74" priority="71" operator="containsText" text="no run">
+      <formula>NOT(ISERROR(SEARCH("no run",E38)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="73" priority="72" operator="containsText" text="blocked">
+      <formula>NOT(ISERROR(SEARCH("blocked",E38)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="72" priority="73" operator="containsText" text="in progres">
+      <formula>NOT(ISERROR(SEARCH("in progres",E38)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="71" priority="74" operator="containsText" text="failed">
+      <formula>NOT(ISERROR(SEARCH("failed",E38)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="70" priority="75" operator="containsText" text="passed">
+      <formula>NOT(ISERROR(SEARCH("passed",E38)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E39">
+    <cfRule type="containsText" dxfId="69" priority="66" operator="containsText" text="no run">
+      <formula>NOT(ISERROR(SEARCH("no run",E39)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="68" priority="67" operator="containsText" text="blocked">
+      <formula>NOT(ISERROR(SEARCH("blocked",E39)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="67" priority="68" operator="containsText" text="in progres">
+      <formula>NOT(ISERROR(SEARCH("in progres",E39)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="66" priority="69" operator="containsText" text="failed">
+      <formula>NOT(ISERROR(SEARCH("failed",E39)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="65" priority="70" operator="containsText" text="passed">
+      <formula>NOT(ISERROR(SEARCH("passed",E39)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E40">
+    <cfRule type="containsText" dxfId="64" priority="61" operator="containsText" text="no run">
+      <formula>NOT(ISERROR(SEARCH("no run",E40)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="63" priority="62" operator="containsText" text="blocked">
+      <formula>NOT(ISERROR(SEARCH("blocked",E40)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="62" priority="63" operator="containsText" text="in progres">
+      <formula>NOT(ISERROR(SEARCH("in progres",E40)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="61" priority="64" operator="containsText" text="failed">
+      <formula>NOT(ISERROR(SEARCH("failed",E40)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="60" priority="65" operator="containsText" text="passed">
+      <formula>NOT(ISERROR(SEARCH("passed",E40)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E41">
+    <cfRule type="containsText" dxfId="59" priority="56" operator="containsText" text="no run">
+      <formula>NOT(ISERROR(SEARCH("no run",E41)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="58" priority="57" operator="containsText" text="blocked">
+      <formula>NOT(ISERROR(SEARCH("blocked",E41)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="57" priority="58" operator="containsText" text="in progres">
+      <formula>NOT(ISERROR(SEARCH("in progres",E41)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="56" priority="59" operator="containsText" text="failed">
+      <formula>NOT(ISERROR(SEARCH("failed",E41)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="55" priority="60" operator="containsText" text="passed">
+      <formula>NOT(ISERROR(SEARCH("passed",E41)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E43">
+    <cfRule type="containsText" dxfId="54" priority="51" operator="containsText" text="no run">
+      <formula>NOT(ISERROR(SEARCH("no run",E43)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="53" priority="52" operator="containsText" text="blocked">
+      <formula>NOT(ISERROR(SEARCH("blocked",E43)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="52" priority="53" operator="containsText" text="in progres">
+      <formula>NOT(ISERROR(SEARCH("in progres",E43)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="51" priority="54" operator="containsText" text="failed">
+      <formula>NOT(ISERROR(SEARCH("failed",E43)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="50" priority="55" operator="containsText" text="passed">
+      <formula>NOT(ISERROR(SEARCH("passed",E43)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E44">
+    <cfRule type="containsText" dxfId="49" priority="46" operator="containsText" text="no run">
+      <formula>NOT(ISERROR(SEARCH("no run",E44)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="48" priority="47" operator="containsText" text="blocked">
+      <formula>NOT(ISERROR(SEARCH("blocked",E44)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="47" priority="48" operator="containsText" text="in progres">
+      <formula>NOT(ISERROR(SEARCH("in progres",E44)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="46" priority="49" operator="containsText" text="failed">
+      <formula>NOT(ISERROR(SEARCH("failed",E44)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="45" priority="50" operator="containsText" text="passed">
+      <formula>NOT(ISERROR(SEARCH("passed",E44)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E45">
+    <cfRule type="containsText" dxfId="44" priority="41" operator="containsText" text="no run">
+      <formula>NOT(ISERROR(SEARCH("no run",E45)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="43" priority="42" operator="containsText" text="blocked">
+      <formula>NOT(ISERROR(SEARCH("blocked",E45)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="42" priority="43" operator="containsText" text="in progres">
+      <formula>NOT(ISERROR(SEARCH("in progres",E45)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="41" priority="44" operator="containsText" text="failed">
+      <formula>NOT(ISERROR(SEARCH("failed",E45)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="40" priority="45" operator="containsText" text="passed">
+      <formula>NOT(ISERROR(SEARCH("passed",E45)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E46">
+    <cfRule type="containsText" dxfId="39" priority="36" operator="containsText" text="no run">
+      <formula>NOT(ISERROR(SEARCH("no run",E46)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="38" priority="37" operator="containsText" text="blocked">
+      <formula>NOT(ISERROR(SEARCH("blocked",E46)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="37" priority="38" operator="containsText" text="in progres">
+      <formula>NOT(ISERROR(SEARCH("in progres",E46)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="36" priority="39" operator="containsText" text="failed">
+      <formula>NOT(ISERROR(SEARCH("failed",E46)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="35" priority="40" operator="containsText" text="passed">
+      <formula>NOT(ISERROR(SEARCH("passed",E46)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E47">
+    <cfRule type="containsText" dxfId="34" priority="31" operator="containsText" text="no run">
+      <formula>NOT(ISERROR(SEARCH("no run",E47)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="33" priority="32" operator="containsText" text="blocked">
+      <formula>NOT(ISERROR(SEARCH("blocked",E47)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="32" priority="33" operator="containsText" text="in progres">
+      <formula>NOT(ISERROR(SEARCH("in progres",E47)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="31" priority="34" operator="containsText" text="failed">
+      <formula>NOT(ISERROR(SEARCH("failed",E47)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="30" priority="35" operator="containsText" text="passed">
+      <formula>NOT(ISERROR(SEARCH("passed",E47)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E48">
+    <cfRule type="containsText" dxfId="29" priority="26" operator="containsText" text="no run">
+      <formula>NOT(ISERROR(SEARCH("no run",E48)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="28" priority="27" operator="containsText" text="blocked">
+      <formula>NOT(ISERROR(SEARCH("blocked",E48)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="27" priority="28" operator="containsText" text="in progres">
+      <formula>NOT(ISERROR(SEARCH("in progres",E48)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="26" priority="29" operator="containsText" text="failed">
+      <formula>NOT(ISERROR(SEARCH("failed",E48)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="25" priority="30" operator="containsText" text="passed">
+      <formula>NOT(ISERROR(SEARCH("passed",E48)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E49">
+    <cfRule type="containsText" dxfId="24" priority="21" operator="containsText" text="no run">
+      <formula>NOT(ISERROR(SEARCH("no run",E49)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="23" priority="22" operator="containsText" text="blocked">
+      <formula>NOT(ISERROR(SEARCH("blocked",E49)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="22" priority="23" operator="containsText" text="in progres">
+      <formula>NOT(ISERROR(SEARCH("in progres",E49)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="21" priority="24" operator="containsText" text="failed">
+      <formula>NOT(ISERROR(SEARCH("failed",E49)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="20" priority="25" operator="containsText" text="passed">
+      <formula>NOT(ISERROR(SEARCH("passed",E49)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E50">
+    <cfRule type="containsText" dxfId="19" priority="16" operator="containsText" text="no run">
+      <formula>NOT(ISERROR(SEARCH("no run",E50)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="18" priority="17" operator="containsText" text="blocked">
+      <formula>NOT(ISERROR(SEARCH("blocked",E50)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="17" priority="18" operator="containsText" text="in progres">
+      <formula>NOT(ISERROR(SEARCH("in progres",E50)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="16" priority="19" operator="containsText" text="failed">
+      <formula>NOT(ISERROR(SEARCH("failed",E50)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="15" priority="20" operator="containsText" text="passed">
+      <formula>NOT(ISERROR(SEARCH("passed",E50)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E51">
+    <cfRule type="containsText" dxfId="14" priority="11" operator="containsText" text="no run">
+      <formula>NOT(ISERROR(SEARCH("no run",E51)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="13" priority="12" operator="containsText" text="blocked">
+      <formula>NOT(ISERROR(SEARCH("blocked",E51)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="12" priority="13" operator="containsText" text="in progres">
+      <formula>NOT(ISERROR(SEARCH("in progres",E51)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="11" priority="14" operator="containsText" text="failed">
+      <formula>NOT(ISERROR(SEARCH("failed",E51)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="10" priority="15" operator="containsText" text="passed">
+      <formula>NOT(ISERROR(SEARCH("passed",E51)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E52">
+    <cfRule type="containsText" dxfId="9" priority="6" operator="containsText" text="no run">
+      <formula>NOT(ISERROR(SEARCH("no run",E52)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="8" priority="7" operator="containsText" text="blocked">
+      <formula>NOT(ISERROR(SEARCH("blocked",E52)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="7" priority="8" operator="containsText" text="in progres">
+      <formula>NOT(ISERROR(SEARCH("in progres",E52)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="6" priority="9" operator="containsText" text="failed">
+      <formula>NOT(ISERROR(SEARCH("failed",E52)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="5" priority="10" operator="containsText" text="passed">
+      <formula>NOT(ISERROR(SEARCH("passed",E52)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E53">
     <cfRule type="containsText" dxfId="4" priority="1" operator="containsText" text="no run">
-      <formula>NOT(ISERROR(SEARCH("no run",E5)))</formula>
+      <formula>NOT(ISERROR(SEARCH("no run",E53)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="blocked">
-      <formula>NOT(ISERROR(SEARCH("blocked",E5)))</formula>
+      <formula>NOT(ISERROR(SEARCH("blocked",E53)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="in progres">
-      <formula>NOT(ISERROR(SEARCH("in progres",E5)))</formula>
+      <formula>NOT(ISERROR(SEARCH("in progres",E53)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="1" priority="4" operator="containsText" text="failed">
-      <formula>NOT(ISERROR(SEARCH("failed",E5)))</formula>
+      <formula>NOT(ISERROR(SEARCH("failed",E53)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="0" priority="5" operator="containsText" text="passed">
-      <formula>NOT(ISERROR(SEARCH("passed",E5)))</formula>
+      <formula>NOT(ISERROR(SEARCH("passed",E53)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
@@ -836,7 +3333,7 @@
           <x14:formula1>
             <xm:f>status!$A$1:$A$5</xm:f>
           </x14:formula1>
-          <xm:sqref>E5:F9</xm:sqref>
+          <xm:sqref>K5:K9 E5:F9 E10:E18 E37:E41 E43:E53</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -847,222 +3344,222 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38B432B5-1BFB-465F-89DC-4FFEFC31F14F}">
   <dimension ref="A1:I14"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="2" max="2" width="36.81640625" customWidth="1"/>
+    <col min="2" max="2" width="36.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="17" x14ac:dyDescent="0.15">
       <c r="A1" s="7">
         <v>1</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="C1" s="20">
+      <c r="C1" s="18">
         <v>1</v>
       </c>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="19"/>
-    </row>
-    <row r="2" spans="1:9" ht="15.5" x14ac:dyDescent="0.25">
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="17"/>
+    </row>
+    <row r="2" spans="1:9" ht="17" x14ac:dyDescent="0.15">
       <c r="A2" s="7">
         <v>2</v>
       </c>
       <c r="B2" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="C2" s="20"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
-      <c r="H2" s="18"/>
-      <c r="I2" s="19"/>
-    </row>
-    <row r="3" spans="1:9" ht="15.5" x14ac:dyDescent="0.25">
+      <c r="C2" s="18"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
+      <c r="I2" s="17"/>
+    </row>
+    <row r="3" spans="1:9" ht="17" x14ac:dyDescent="0.15">
       <c r="A3" s="7">
         <v>3</v>
       </c>
       <c r="B3" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
-      <c r="G3" s="18"/>
-      <c r="H3" s="18"/>
-      <c r="I3" s="19"/>
-    </row>
-    <row r="4" spans="1:9" ht="15.5" x14ac:dyDescent="0.25">
+      <c r="C3" s="18"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="16"/>
+      <c r="G3" s="16"/>
+      <c r="H3" s="16"/>
+      <c r="I3" s="17"/>
+    </row>
+    <row r="4" spans="1:9" ht="17" x14ac:dyDescent="0.15">
       <c r="A4" s="7">
         <v>4</v>
       </c>
       <c r="B4" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="20"/>
-      <c r="D4" s="18"/>
-      <c r="E4" s="18"/>
-      <c r="F4" s="18"/>
-      <c r="G4" s="18"/>
-      <c r="H4" s="18"/>
-      <c r="I4" s="19"/>
-    </row>
-    <row r="5" spans="1:9" ht="15.5" x14ac:dyDescent="0.25">
+      <c r="C4" s="18"/>
+      <c r="D4" s="16"/>
+      <c r="E4" s="16"/>
+      <c r="F4" s="16"/>
+      <c r="G4" s="16"/>
+      <c r="H4" s="16"/>
+      <c r="I4" s="17"/>
+    </row>
+    <row r="5" spans="1:9" ht="17" x14ac:dyDescent="0.15">
       <c r="A5" s="7">
         <v>5</v>
       </c>
       <c r="B5" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="20"/>
-      <c r="D5" s="18"/>
-      <c r="E5" s="18"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18"/>
-      <c r="H5" s="18"/>
-      <c r="I5" s="19"/>
-    </row>
-    <row r="6" spans="1:9" ht="15.5" x14ac:dyDescent="0.25">
+      <c r="C5" s="18"/>
+      <c r="D5" s="16"/>
+      <c r="E5" s="16"/>
+      <c r="F5" s="16"/>
+      <c r="G5" s="16"/>
+      <c r="H5" s="16"/>
+      <c r="I5" s="17"/>
+    </row>
+    <row r="6" spans="1:9" ht="17" x14ac:dyDescent="0.15">
       <c r="A6" s="7">
         <v>6</v>
       </c>
       <c r="B6" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="20"/>
-      <c r="D6" s="18"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="18"/>
-      <c r="H6" s="18"/>
-      <c r="I6" s="19"/>
-    </row>
-    <row r="7" spans="1:9" ht="15.5" x14ac:dyDescent="0.25">
+      <c r="C6" s="18"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="16"/>
+      <c r="H6" s="16"/>
+      <c r="I6" s="17"/>
+    </row>
+    <row r="7" spans="1:9" ht="17" x14ac:dyDescent="0.15">
       <c r="A7" s="7">
         <v>7</v>
       </c>
       <c r="B7" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="20"/>
-      <c r="D7" s="18"/>
-      <c r="E7" s="18"/>
-      <c r="F7" s="18"/>
-      <c r="G7" s="18"/>
-      <c r="H7" s="18"/>
-      <c r="I7" s="19"/>
-    </row>
-    <row r="8" spans="1:9" ht="31" x14ac:dyDescent="0.25">
+      <c r="C7" s="18"/>
+      <c r="D7" s="16"/>
+      <c r="E7" s="16"/>
+      <c r="F7" s="16"/>
+      <c r="G7" s="16"/>
+      <c r="H7" s="16"/>
+      <c r="I7" s="17"/>
+    </row>
+    <row r="8" spans="1:9" ht="34" x14ac:dyDescent="0.15">
       <c r="A8" s="7">
         <v>8</v>
       </c>
       <c r="B8" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="C8" s="20"/>
-      <c r="D8" s="18"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18"/>
-      <c r="G8" s="18"/>
-      <c r="H8" s="18"/>
-      <c r="I8" s="19"/>
-    </row>
-    <row r="9" spans="1:9" ht="15.5" x14ac:dyDescent="0.25">
+      <c r="C8" s="18"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="16"/>
+      <c r="G8" s="16"/>
+      <c r="H8" s="16"/>
+      <c r="I8" s="17"/>
+    </row>
+    <row r="9" spans="1:9" ht="17" x14ac:dyDescent="0.15">
       <c r="A9" s="7">
         <v>9</v>
       </c>
       <c r="B9" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="20"/>
-      <c r="D9" s="18"/>
-      <c r="E9" s="18"/>
-      <c r="F9" s="18"/>
-      <c r="G9" s="18"/>
-      <c r="H9" s="18"/>
-      <c r="I9" s="19"/>
-    </row>
-    <row r="10" spans="1:9" ht="15.5" x14ac:dyDescent="0.25">
+      <c r="C9" s="18"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="16"/>
+      <c r="G9" s="16"/>
+      <c r="H9" s="16"/>
+      <c r="I9" s="17"/>
+    </row>
+    <row r="10" spans="1:9" ht="17" x14ac:dyDescent="0.15">
       <c r="A10" s="7">
         <v>10</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="18"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="18"/>
-      <c r="G10" s="18"/>
-      <c r="H10" s="18"/>
-      <c r="I10" s="19"/>
-    </row>
-    <row r="11" spans="1:9" ht="15.5" x14ac:dyDescent="0.25">
+      <c r="C10" s="16"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="16"/>
+      <c r="G10" s="16"/>
+      <c r="H10" s="16"/>
+      <c r="I10" s="17"/>
+    </row>
+    <row r="11" spans="1:9" ht="17" x14ac:dyDescent="0.15">
       <c r="A11" s="7">
         <v>11</v>
       </c>
       <c r="B11" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="18"/>
-      <c r="D11" s="18"/>
-      <c r="E11" s="18"/>
-      <c r="F11" s="18"/>
-      <c r="G11" s="18"/>
-      <c r="H11" s="18"/>
-      <c r="I11" s="19"/>
-    </row>
-    <row r="12" spans="1:9" ht="15.5" x14ac:dyDescent="0.25">
+      <c r="C11" s="16"/>
+      <c r="D11" s="16"/>
+      <c r="E11" s="16"/>
+      <c r="F11" s="16"/>
+      <c r="G11" s="16"/>
+      <c r="H11" s="16"/>
+      <c r="I11" s="17"/>
+    </row>
+    <row r="12" spans="1:9" ht="17" x14ac:dyDescent="0.15">
       <c r="A12" s="7">
         <v>12</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="18"/>
-      <c r="D12" s="18"/>
-      <c r="E12" s="18"/>
-      <c r="F12" s="18"/>
-      <c r="G12" s="18"/>
-      <c r="H12" s="18"/>
-      <c r="I12" s="19"/>
-    </row>
-    <row r="13" spans="1:9" ht="15.5" x14ac:dyDescent="0.25">
+      <c r="C12" s="16"/>
+      <c r="D12" s="16"/>
+      <c r="E12" s="16"/>
+      <c r="F12" s="16"/>
+      <c r="G12" s="16"/>
+      <c r="H12" s="16"/>
+      <c r="I12" s="17"/>
+    </row>
+    <row r="13" spans="1:9" ht="17" x14ac:dyDescent="0.15">
       <c r="A13" s="7">
         <v>13</v>
       </c>
       <c r="B13" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="C13" s="20"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="18"/>
-      <c r="F13" s="18"/>
-      <c r="G13" s="18"/>
-      <c r="H13" s="18"/>
-      <c r="I13" s="19"/>
-    </row>
-    <row r="14" spans="1:9" ht="15.5" x14ac:dyDescent="0.25">
+      <c r="C13" s="18"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="16"/>
+      <c r="F13" s="16"/>
+      <c r="G13" s="16"/>
+      <c r="H13" s="16"/>
+      <c r="I13" s="17"/>
+    </row>
+    <row r="14" spans="1:9" ht="17" x14ac:dyDescent="0.15">
       <c r="A14" s="7">
         <v>14</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="C14" s="18"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
-      <c r="F14" s="18"/>
-      <c r="G14" s="18"/>
-      <c r="H14" s="18"/>
-      <c r="I14" s="19"/>
+      <c r="C14" s="16"/>
+      <c r="D14" s="16"/>
+      <c r="E14" s="16"/>
+      <c r="F14" s="16"/>
+      <c r="G14" s="16"/>
+      <c r="H14" s="16"/>
+      <c r="I14" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="14">
@@ -1089,29 +3586,29 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1B46851-6ED7-4089-8D23-0B2B6990E1E3}">
   <dimension ref="A1:A5"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A2" s="5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A3" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A4" s="4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A5" s="3" t="s">
         <v>11</v>
       </c>
@@ -1124,77 +3621,10 @@
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10001</Type>
-    <SequenceNumber>1000</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10002</Type>
-    <SequenceNumber>1001</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10004</Type>
-    <SequenceNumber>1002</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10006</Type>
-    <SequenceNumber>1003</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-</spe:Receivers>
+<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="34c87397-5fc1-491e-85e7-d6110dbe9cbd" ContentTypeId="0x0101" PreviousValue="false"/>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <HideFromDelve xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105">false</HideFromDelve>
-    <_dlc_DocId xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105">S5IOPQAIPMN3-1127675540-13</_dlc_DocId>
-    <_dlc_DocIdUrl xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105">
-      <Url>https://nokia.sharepoint.com/sites/TestowanieOprogramowaniaNS/_layouts/15/DocIdRedir.aspx?ID=S5IOPQAIPMN3-1127675540-13</Url>
-      <Description>S5IOPQAIPMN3-1127675540-13</Description>
-    </_dlc_DocIdUrl>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100112D85FF5A30B44EAC277C80404B7C3F" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="921af60d48d10d6d782bdb702f9d8b77">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="71c5aaf6-e6ce-465b-b873-5148d2a4c105" xmlns:ns3="66745ed6-1243-4599-9e8d-d86d6e083497" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="45c3cf35de4cdcc6ced4e5381f09f675" ns2:_="" ns3:_="">
     <xsd:import namespace="71c5aaf6-e6ce-465b-b873-5148d2a4c105"/>
@@ -1392,20 +3822,114 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <HideFromDelve xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105">false</HideFromDelve>
+    <_dlc_DocId xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105">S5IOPQAIPMN3-1127675540-13</_dlc_DocId>
+    <_dlc_DocIdUrl xmlns="71c5aaf6-e6ce-465b-b873-5148d2a4c105">
+      <Url>https://nokia.sharepoint.com/sites/TestowanieOprogramowaniaNS/_layouts/15/DocIdRedir.aspx?ID=S5IOPQAIPMN3-1127675540-13</Url>
+      <Description>S5IOPQAIPMN3-1127675540-13</Description>
+    </_dlc_DocIdUrl>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
-<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="34c87397-5fc1-491e-85e7-d6110dbe9cbd" ContentTypeId="0x0101" PreviousValue="false"/>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{27815257-2363-4D78-BB28-2D8BE4BFCA9C}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9443A8EE-7C88-42CE-B936-1663D159B01C}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
+    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{326B8469-24AF-4FAF-B1BB-FDEDFAA19DE7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="71c5aaf6-e6ce-465b-b873-5148d2a4c105"/>
+    <ds:schemaRef ds:uri="66745ed6-1243-4599-9e8d-d86d6e083497"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5236D923-EA41-4A5F-B46A-4D66CC1D6C71}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AECCC26E-DF35-47CA-AC84-400530547BBB}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
@@ -1423,22 +3947,10 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5236D923-EA41-4A5F-B46A-4D66CC1D6C71}">
+<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{27815257-2363-4D78-BB28-2D8BE4BFCA9C}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{326B8469-24AF-4FAF-B1BB-FDEDFAA19DE7}"/>
-</file>
-
-<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9443A8EE-7C88-42CE-B936-1663D159B01C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>